<commit_message>
fix: wrong column reference in the manual for the reference value optimizer
</commit_message>
<xml_diff>
--- a/Subjective bias of criteria aggregation/Reference value optimizer.xlsx
+++ b/Subjective bias of criteria aggregation/Reference value optimizer.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr codeName="Ten_skoroszyt" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tomash/Articles/2025Evaluation-RP/aggregation/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tomash/Projects/DesignFlawsEvaluation/Subjective bias of criteria aggregation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1239E95-1B23-0142-8CDE-1508C943F1C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAC4D9BC-3201-D343-BE51-93C393ECDABC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20560" yWindow="880" windowWidth="20560" windowHeight="25700" xr2:uid="{9E4405CB-EE6D-D946-B9BD-19404967C641}"/>
+    <workbookView xWindow="20580" yWindow="880" windowWidth="20560" windowHeight="25700" xr2:uid="{9E4405CB-EE6D-D946-B9BD-19404967C641}"/>
   </bookViews>
   <sheets>
     <sheet name="simulation" sheetId="4" r:id="rId1"/>
@@ -68,7 +68,7 @@
     <definedName name="solver_val" localSheetId="0" hidden="1">0</definedName>
     <definedName name="solver_ver" localSheetId="0" hidden="1">2</definedName>
   </definedNames>
-  <calcPr calcId="191029" calcMode="manual"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -160,7 +160,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="82">
   <si>
     <t>N</t>
   </si>
@@ -399,10 +399,13 @@
     <t>AJP</t>
   </si>
   <si>
-    <t>1. Set the desired categories in S column; leave cell empty if unspecified</t>
-  </si>
-  <si>
     <t>Initial category</t>
+  </si>
+  <si>
+    <t>1. Set the desired categories in the Desired category column; leave cell empty if unspecified</t>
+  </si>
+  <si>
+    <t>Calculated reference values:</t>
   </si>
 </sst>
 </file>
@@ -468,15 +471,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normalny" xfId="0" builtinId="0"/>
@@ -816,7 +817,7 @@
   <dimension ref="A1:X66"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="39.6640625" customWidth="1"/>
+    <col min="1" max="1" width="67.5" customWidth="1"/>
     <col min="2" max="2" width="25.5" customWidth="1"/>
     <col min="6" max="6" width="10.83203125" customWidth="1"/>
     <col min="7" max="9" width="10.83203125" hidden="1" customWidth="1"/>
@@ -848,7 +849,7 @@
     </row>
     <row r="2" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B2" t="s">
         <v>28</v>
@@ -862,14 +863,14 @@
       <c r="E2" s="2">
         <v>75.873000000000005</v>
       </c>
-      <c r="T2" s="6">
+      <c r="T2" s="5">
         <f t="array" ref="T2:V4">(C7:E9-C2:E4)/C2:E4</f>
         <v>1.9735911127771691E-2</v>
       </c>
-      <c r="U2" s="6">
+      <c r="U2" s="5">
         <v>-0.58407005034566251</v>
       </c>
-      <c r="V2" s="6">
+      <c r="V2" s="5">
         <v>-1.2540393358810334E-2</v>
       </c>
     </row>
@@ -886,13 +887,13 @@
       <c r="E3" s="2">
         <v>51.15</v>
       </c>
-      <c r="T3" s="6">
+      <c r="T3" s="5">
         <v>0.50667202722292737</v>
       </c>
-      <c r="U3" s="6">
+      <c r="U3" s="5">
         <v>-0.39254959733739059</v>
       </c>
-      <c r="V3" s="6">
+      <c r="V3" s="5">
         <v>2.5856934681634395E-3</v>
       </c>
     </row>
@@ -909,18 +910,18 @@
       <c r="E4" s="2">
         <v>34.1</v>
       </c>
-      <c r="T4" s="6">
+      <c r="T4" s="5">
         <v>2.9145733838442378E-3</v>
       </c>
-      <c r="U4" s="7">
+      <c r="U4" s="5">
         <v>-0.1025975392203146</v>
       </c>
-      <c r="V4" s="6">
+      <c r="V4" s="5">
         <v>-1.9908730779541855E-4</v>
       </c>
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="4" t="s">
         <v>40</v>
       </c>
       <c r="B5" t="s">
@@ -931,6 +932,9 @@
       </c>
     </row>
     <row r="6" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="B6" t="s">
+        <v>81</v>
+      </c>
       <c r="C6" t="s">
         <v>12</v>
       </c>
@@ -1005,13 +1009,13 @@
       <c r="B10" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="4">
+      <c r="C10" s="2">
         <v>50</v>
       </c>
-      <c r="D10" s="4">
+      <c r="D10" s="2">
         <v>35</v>
       </c>
-      <c r="E10" s="4">
+      <c r="E10" s="2">
         <v>15</v>
       </c>
       <c r="X10" s="1">
@@ -1075,7 +1079,7 @@
         <v>9</v>
       </c>
       <c r="S11" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="T11" t="s">
         <v>32</v>
@@ -1125,7 +1129,7 @@
         <v>-0.48529570746621453</v>
       </c>
       <c r="J12" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,G12:I12)</f>
+        <f t="shared" ref="J12:J50" si="0">SUMPRODUCT($C$10:$E$10,G12:I12)</f>
         <v>77.720564388006778</v>
       </c>
       <c r="K12" s="1" cm="1">
@@ -1141,7 +1145,7 @@
         <v>0.96195254991002788</v>
       </c>
       <c r="N12" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,K12:M12)</f>
+        <f t="shared" ref="N12:N50" si="1">SUMPRODUCT($C$10:$E$10,K12:M12)</f>
         <v>99.429288248650423</v>
       </c>
       <c r="O12" s="1" cm="1">
@@ -1157,7 +1161,7 @@
         <v>1</v>
       </c>
       <c r="R12" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,O12:Q12)</f>
+        <f t="shared" ref="R12:R50" si="2">SUMPRODUCT($C$10:$E$10,O12:Q12)</f>
         <v>100</v>
       </c>
       <c r="S12" s="1" t="s">
@@ -1177,7 +1181,7 @@
         <v>1</v>
       </c>
       <c r="X12" s="1">
-        <f>ABS(V12-W12)^1.5</f>
+        <f t="shared" ref="X12:X50" si="3">ABS(V12-W12)^1.5</f>
         <v>0</v>
       </c>
     </row>
@@ -1213,7 +1217,7 @@
         <v>0.15431641571387011</v>
       </c>
       <c r="J13" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,G13:I13)</f>
+        <f t="shared" si="0"/>
         <v>76.945302121293309</v>
       </c>
       <c r="K13" s="1" cm="1">
@@ -1229,7 +1233,7 @@
         <v>1</v>
       </c>
       <c r="N13" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,K13:M13)</f>
+        <f t="shared" si="1"/>
         <v>90.375672817856127</v>
       </c>
       <c r="O13" s="1" cm="1">
@@ -1245,7 +1249,7 @@
         <v>1</v>
       </c>
       <c r="R13" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,O13:Q13)</f>
+        <f t="shared" si="2"/>
         <v>100</v>
       </c>
       <c r="S13" s="1" t="s">
@@ -1265,7 +1269,7 @@
         <v>1</v>
       </c>
       <c r="X13" s="1">
-        <f>ABS(V13-W13)^1.5</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -1301,7 +1305,7 @@
         <v>-0.26032231499243685</v>
       </c>
       <c r="J14" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,G14:I14)</f>
+        <f t="shared" si="0"/>
         <v>69.526961824421093</v>
       </c>
       <c r="K14" s="1" cm="1">
@@ -1317,7 +1321,7 @@
         <v>1</v>
       </c>
       <c r="N14" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,K14:M14)</f>
+        <f t="shared" si="1"/>
         <v>89.177397838009298</v>
       </c>
       <c r="O14" s="1" cm="1">
@@ -1333,7 +1337,7 @@
         <v>1</v>
       </c>
       <c r="R14" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,O14:Q14)</f>
+        <f t="shared" si="2"/>
         <v>100</v>
       </c>
       <c r="S14" s="1" t="s">
@@ -1353,7 +1357,7 @@
         <v>1</v>
       </c>
       <c r="X14" s="1">
-        <f>ABS(V14-W14)^1.5</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -1389,7 +1393,7 @@
         <v>-1</v>
       </c>
       <c r="J15" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,G15:I15)</f>
+        <f t="shared" si="0"/>
         <v>58.431796549307649</v>
       </c>
       <c r="K15" s="1" cm="1">
@@ -1405,7 +1409,7 @@
         <v>-1</v>
       </c>
       <c r="N15" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,K15:M15)</f>
+        <f t="shared" si="1"/>
         <v>59.177397838009298</v>
       </c>
       <c r="O15" s="1" cm="1">
@@ -1421,7 +1425,7 @@
         <v>-0.48954983177439149</v>
       </c>
       <c r="R15" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,O15:Q15)</f>
+        <f t="shared" si="2"/>
         <v>77.656752523384128</v>
       </c>
       <c r="S15" s="1" t="s">
@@ -1441,7 +1445,7 @@
         <v>1</v>
       </c>
       <c r="X15" s="1">
-        <f>ABS(V15-W15)^1.5</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -1477,7 +1481,7 @@
         <v>0.25128498918581443</v>
       </c>
       <c r="J16" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,G16:I16)</f>
+        <f t="shared" si="0"/>
         <v>50.408774817968606</v>
       </c>
       <c r="K16" s="1" cm="1">
@@ -1493,7 +1497,7 @@
         <v>1</v>
       </c>
       <c r="N16" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,K16:M16)</f>
+        <f t="shared" si="1"/>
         <v>62.392082683613168</v>
       </c>
       <c r="O16" s="1" cm="1">
@@ -1509,7 +1513,7 @@
         <v>1</v>
       </c>
       <c r="R16" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,O16:Q16)</f>
+        <f t="shared" si="2"/>
         <v>100</v>
       </c>
       <c r="S16" s="1" t="s">
@@ -1529,7 +1533,7 @@
         <v>1</v>
       </c>
       <c r="X16" s="1">
-        <f>ABS(V16-W16)^1.5</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -1565,7 +1569,7 @@
         <v>1</v>
       </c>
       <c r="J17" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,G17:I17)</f>
+        <f t="shared" si="0"/>
         <v>49.995167491387846</v>
       </c>
       <c r="K17" s="1" cm="1">
@@ -1581,7 +1585,7 @@
         <v>1</v>
       </c>
       <c r="N17" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,K17:M17)</f>
+        <f t="shared" si="1"/>
         <v>50.748489869555243</v>
       </c>
       <c r="O17" s="1" cm="1">
@@ -1597,7 +1601,7 @@
         <v>1</v>
       </c>
       <c r="R17" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,O17:Q17)</f>
+        <f t="shared" si="2"/>
         <v>100</v>
       </c>
       <c r="S17" s="1" t="s">
@@ -1617,7 +1621,7 @@
         <v>1</v>
       </c>
       <c r="X17" s="1">
-        <f>ABS(V17-W17)^1.5</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -1653,7 +1657,7 @@
         <v>0.43790013932499083</v>
       </c>
       <c r="J18" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,G18:I18)</f>
+        <f t="shared" si="0"/>
         <v>48.643199769912485</v>
       </c>
       <c r="K18" s="1" cm="1">
@@ -1669,7 +1673,7 @@
         <v>1</v>
       </c>
       <c r="N18" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,K18:M18)</f>
+        <f t="shared" si="1"/>
         <v>57.827736054704971</v>
       </c>
       <c r="O18" s="1" cm="1">
@@ -1685,7 +1689,7 @@
         <v>1</v>
       </c>
       <c r="R18" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,O18:Q18)</f>
+        <f t="shared" si="2"/>
         <v>100</v>
       </c>
       <c r="S18" s="1" t="s">
@@ -1705,7 +1709,7 @@
         <v>1</v>
       </c>
       <c r="X18" s="1">
-        <f>ABS(V18-W18)^1.5</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -1741,7 +1745,7 @@
         <v>-0.66258939212270285</v>
       </c>
       <c r="J19" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,G19:I19)</f>
+        <f t="shared" si="0"/>
         <v>40.706397876653597</v>
       </c>
       <c r="K19" s="1" cm="1">
@@ -1757,7 +1761,7 @@
         <v>0.78597711417734262</v>
       </c>
       <c r="N19" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,K19:M19)</f>
+        <f t="shared" si="1"/>
         <v>63.18690228984461</v>
       </c>
       <c r="O19" s="1" cm="1">
@@ -1773,7 +1777,7 @@
         <v>1</v>
       </c>
       <c r="R19" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,O19:Q19)</f>
+        <f t="shared" si="2"/>
         <v>100</v>
       </c>
       <c r="S19" s="1" t="s">
@@ -1793,7 +1797,7 @@
         <v>1</v>
       </c>
       <c r="X19" s="1">
-        <f>ABS(V19-W19)^1.5</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -1829,7 +1833,7 @@
         <v>0.3690308162425413</v>
       </c>
       <c r="J20" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,G20:I20)</f>
+        <f t="shared" si="0"/>
         <v>40.560831521986231</v>
       </c>
       <c r="K20" s="1" cm="1">
@@ -1845,7 +1849,7 @@
         <v>1</v>
       </c>
       <c r="N20" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,K20:M20)</f>
+        <f t="shared" si="1"/>
         <v>50.778691536663388</v>
       </c>
       <c r="O20" s="1" cm="1">
@@ -1861,7 +1865,7 @@
         <v>1</v>
       </c>
       <c r="R20" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,O20:Q20)</f>
+        <f t="shared" si="2"/>
         <v>100</v>
       </c>
       <c r="S20" s="1" t="s">
@@ -1881,7 +1885,7 @@
         <v>1</v>
       </c>
       <c r="X20" s="1">
-        <f>ABS(V20-W20)^1.5</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -1917,7 +1921,7 @@
         <v>-0.15242936489198133</v>
       </c>
       <c r="J21" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,G21:I21)</f>
+        <f t="shared" si="0"/>
         <v>40.387968554535739</v>
       </c>
       <c r="K21" s="1" cm="1">
@@ -1933,7 +1937,7 @@
         <v>1</v>
       </c>
       <c r="N21" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,K21:M21)</f>
+        <f t="shared" si="1"/>
         <v>60.486514029574934</v>
       </c>
       <c r="O21" s="1" cm="1">
@@ -1949,7 +1953,7 @@
         <v>1</v>
       </c>
       <c r="R21" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,O21:Q21)</f>
+        <f t="shared" si="2"/>
         <v>98.400800696790483</v>
       </c>
       <c r="S21" s="1" t="s">
@@ -1969,7 +1973,7 @@
         <v>1</v>
       </c>
       <c r="X21" s="1">
-        <f>ABS(V21-W21)^1.5</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -2005,7 +2009,7 @@
         <v>-0.48529570746621453</v>
       </c>
       <c r="J22" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,G22:I22)</f>
+        <f t="shared" si="0"/>
         <v>31.080873386672966</v>
       </c>
       <c r="K22" s="1" cm="1">
@@ -2021,7 +2025,7 @@
         <v>0.96195254991002788</v>
       </c>
       <c r="N22" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,K22:M22)</f>
+        <f t="shared" si="1"/>
         <v>53.542848722910605</v>
       </c>
       <c r="O22" s="1" cm="1">
@@ -2037,7 +2041,7 @@
         <v>1</v>
       </c>
       <c r="R22" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,O22:Q22)</f>
+        <f t="shared" si="2"/>
         <v>100</v>
       </c>
       <c r="S22" s="1" t="s">
@@ -2057,7 +2061,7 @@
         <v>1</v>
       </c>
       <c r="X22" s="1">
-        <f>ABS(V22-W22)^1.5</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -2093,7 +2097,7 @@
         <v>0.48309528055824269</v>
       </c>
       <c r="J23" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,G23:I23)</f>
+        <f t="shared" si="0"/>
         <v>30.030585589821371</v>
       </c>
       <c r="K23" s="1" cm="1">
@@ -2109,7 +2113,7 @@
         <v>1</v>
       </c>
       <c r="N23" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,K23:M23)</f>
+        <f t="shared" si="1"/>
         <v>38.536760645751997</v>
       </c>
       <c r="O23" s="1" cm="1">
@@ -2125,7 +2129,7 @@
         <v>1</v>
       </c>
       <c r="R23" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,O23:Q23)</f>
+        <f t="shared" si="2"/>
         <v>100</v>
       </c>
       <c r="S23" s="1" t="s">
@@ -2145,7 +2149,7 @@
         <v>1</v>
       </c>
       <c r="X23" s="1">
-        <f>ABS(V23-W23)^1.5</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -2181,7 +2185,7 @@
         <v>1</v>
       </c>
       <c r="J24" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,G24:I24)</f>
+        <f t="shared" si="0"/>
         <v>26.824597839293951</v>
       </c>
       <c r="K24" s="1" cm="1">
@@ -2197,7 +2201,7 @@
         <v>1</v>
       </c>
       <c r="N24" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,K24:M24)</f>
+        <f t="shared" si="1"/>
         <v>27.575255144640852</v>
       </c>
       <c r="O24" s="1" cm="1">
@@ -2213,7 +2217,7 @@
         <v>1</v>
       </c>
       <c r="R24" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,O24:Q24)</f>
+        <f t="shared" si="2"/>
         <v>100</v>
       </c>
       <c r="S24" s="1" t="s">
@@ -2233,7 +2237,7 @@
         <v>1</v>
       </c>
       <c r="X24" s="1">
-        <f>ABS(V24-W24)^1.5</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -2269,7 +2273,7 @@
         <v>-1</v>
       </c>
       <c r="J25" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,G25:I25)</f>
+        <f t="shared" si="0"/>
         <v>23.864134077873082</v>
       </c>
       <c r="K25" s="1" cm="1">
@@ -2285,7 +2289,7 @@
         <v>-1</v>
       </c>
       <c r="N25" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,K25:M25)</f>
+        <f t="shared" si="1"/>
         <v>24.617364942429823</v>
       </c>
       <c r="O25" s="1" cm="1">
@@ -2301,7 +2305,7 @@
         <v>-0.1833952838921975</v>
       </c>
       <c r="R25" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,O25:Q25)</f>
+        <f t="shared" si="2"/>
         <v>82.249070741617032</v>
       </c>
       <c r="S25" s="1" t="s">
@@ -2321,7 +2325,7 @@
         <v>1</v>
       </c>
       <c r="X25" s="1">
-        <f>ABS(V25-W25)^1.5</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -2357,7 +2361,7 @@
         <v>-1</v>
       </c>
       <c r="J26" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,G26:I26)</f>
+        <f t="shared" si="0"/>
         <v>22.723412522193222</v>
       </c>
       <c r="K26" s="1" cm="1">
@@ -2373,7 +2377,7 @@
         <v>-0.50016616136474634</v>
       </c>
       <c r="N26" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,K26:M26)</f>
+        <f t="shared" si="1"/>
         <v>33.046899760479491</v>
       </c>
       <c r="O26" s="1" cm="1">
@@ -2389,7 +2393,7 @@
         <v>1</v>
       </c>
       <c r="R26" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,O26:Q26)</f>
+        <f t="shared" si="2"/>
         <v>59.509869472567459</v>
       </c>
       <c r="S26" s="1" t="s">
@@ -2409,7 +2413,7 @@
         <v>1</v>
       </c>
       <c r="X26" s="1">
-        <f>ABS(V26-W26)^1.5</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -2445,7 +2449,7 @@
         <v>-1</v>
       </c>
       <c r="J27" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,G27:I27)</f>
+        <f t="shared" si="0"/>
         <v>11.227132275927669</v>
       </c>
       <c r="K27" s="1" cm="1">
@@ -2461,7 +2465,7 @@
         <v>0.26814100895797655</v>
       </c>
       <c r="N27" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,K27:M27)</f>
+        <f t="shared" si="1"/>
         <v>31.002208973565729</v>
       </c>
       <c r="O27" s="1" cm="1">
@@ -2477,7 +2481,7 @@
         <v>1</v>
       </c>
       <c r="R27" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,O27:Q27)</f>
+        <f t="shared" si="2"/>
         <v>100</v>
       </c>
       <c r="S27" s="1" t="s">
@@ -2497,7 +2501,7 @@
         <v>1</v>
       </c>
       <c r="X27" s="1">
-        <f>ABS(V27-W27)^1.5</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -2533,7 +2537,7 @@
         <v>-1</v>
       </c>
       <c r="J28" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,G28:I28)</f>
+        <f t="shared" si="0"/>
         <v>9.0654366352171714</v>
       </c>
       <c r="K28" s="1" cm="1">
@@ -2549,7 +2553,7 @@
         <v>-1</v>
       </c>
       <c r="N28" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,K28:M28)</f>
+        <f t="shared" si="1"/>
         <v>11.133925091069496</v>
       </c>
       <c r="O28" s="1" cm="1">
@@ -2565,7 +2569,7 @@
         <v>-0.48954983177439149</v>
       </c>
       <c r="R28" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,O28:Q28)</f>
+        <f t="shared" si="2"/>
         <v>20.819073589292735</v>
       </c>
       <c r="S28" s="1" t="s">
@@ -2585,7 +2589,7 @@
         <v>1</v>
       </c>
       <c r="X28" s="1">
-        <f>ABS(V28-W28)^1.5</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -2621,7 +2625,7 @@
         <v>0.25128498918581443</v>
       </c>
       <c r="J29" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,G29:I29)</f>
+        <f t="shared" si="0"/>
         <v>1.006164591293798</v>
       </c>
       <c r="K29" s="1" cm="1">
@@ -2637,7 +2641,7 @@
         <v>1</v>
       </c>
       <c r="N29" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,K29:M29)</f>
+        <f t="shared" si="1"/>
         <v>15.057182196965954</v>
       </c>
       <c r="O29" s="1" cm="1">
@@ -2653,7 +2657,7 @@
         <v>1</v>
       </c>
       <c r="R29" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,O29:Q29)</f>
+        <f t="shared" si="2"/>
         <v>91.754234833383862</v>
       </c>
       <c r="S29" s="1" t="s">
@@ -2675,7 +2679,7 @@
         <v>1</v>
       </c>
       <c r="X29" s="1">
-        <f>ABS(V29-W29)^1.5</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -2711,7 +2715,7 @@
         <v>-1</v>
       </c>
       <c r="J30" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,G30:I30)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="K30" s="1" cm="1">
@@ -2727,7 +2731,7 @@
         <v>-1</v>
       </c>
       <c r="N30" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,K30:M30)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="O30" s="1" cm="1">
@@ -2743,7 +2747,7 @@
         <v>-1</v>
       </c>
       <c r="R30" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,O30:Q30)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="S30" s="1" t="s">
@@ -2763,7 +2767,7 @@
         <v>1</v>
       </c>
       <c r="X30" s="1">
-        <f>ABS(V30-W30)^1.5</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -2799,7 +2803,7 @@
         <v>-0.66258939212270285</v>
       </c>
       <c r="J31" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,G31:I31)</f>
+        <f t="shared" si="0"/>
         <v>-1.1461145469384295</v>
       </c>
       <c r="K31" s="1" cm="1">
@@ -2815,7 +2819,7 @@
         <v>0.78597711417734262</v>
       </c>
       <c r="N31" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,K31:M31)</f>
+        <f t="shared" si="1"/>
         <v>21.332284142372021</v>
       </c>
       <c r="O31" s="1" cm="1">
@@ -2831,7 +2835,7 @@
         <v>1</v>
       </c>
       <c r="R31" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,O31:Q31)</f>
+        <f t="shared" si="2"/>
         <v>100</v>
       </c>
       <c r="S31" s="1" t="s">
@@ -2851,7 +2855,7 @@
         <v>2</v>
       </c>
       <c r="X31" s="1">
-        <f>ABS(V31-W31)^1.5</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -2887,7 +2891,7 @@
         <v>-1</v>
       </c>
       <c r="J32" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,G32:I32)</f>
+        <f t="shared" si="0"/>
         <v>-5.3404081124193112</v>
       </c>
       <c r="K32" s="1" cm="1">
@@ -2903,7 +2907,7 @@
         <v>-1</v>
       </c>
       <c r="N32" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,K32:M32)</f>
+        <f t="shared" si="1"/>
         <v>-4.5974836601039328</v>
       </c>
       <c r="O32" s="1" cm="1">
@@ -2919,7 +2923,7 @@
         <v>-1</v>
       </c>
       <c r="R32" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,O32:Q32)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="S32" s="1" t="s">
@@ -2939,7 +2943,7 @@
         <v>3</v>
       </c>
       <c r="X32" s="1">
-        <f>ABS(V32-W32)^1.5</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -2975,7 +2979,7 @@
         <v>-0.23307085278966289</v>
       </c>
       <c r="J33" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,G33:I33)</f>
+        <f t="shared" si="0"/>
         <v>-17.041920846098868</v>
       </c>
       <c r="K33" s="1" cm="1">
@@ -2991,7 +2995,7 @@
         <v>1</v>
       </c>
       <c r="N33" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,K33:M33)</f>
+        <f t="shared" si="1"/>
         <v>2.2050213607952287</v>
       </c>
       <c r="O33" s="1" cm="1">
@@ -3007,7 +3011,7 @@
         <v>1</v>
       </c>
       <c r="R33" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,O33:Q33)</f>
+        <f t="shared" si="2"/>
         <v>30</v>
       </c>
       <c r="S33" s="1" t="s">
@@ -3027,7 +3031,7 @@
         <v>2</v>
       </c>
       <c r="X33" s="1">
-        <f>ABS(V33-W33)^1.5</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -3063,7 +3067,7 @@
         <v>-0.17912627790187374</v>
       </c>
       <c r="J34" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,G34:I34)</f>
+        <f t="shared" si="0"/>
         <v>-17.686894168528106</v>
       </c>
       <c r="K34" s="1" cm="1">
@@ -3079,7 +3083,7 @@
         <v>1</v>
       </c>
       <c r="N34" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,K34:M34)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="O34" s="1" cm="1">
@@ -3095,7 +3099,7 @@
         <v>1</v>
       </c>
       <c r="R34" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,O34:Q34)</f>
+        <f t="shared" si="2"/>
         <v>94.690460608543816</v>
       </c>
       <c r="S34" s="1" t="s">
@@ -3115,7 +3119,7 @@
         <v>2</v>
       </c>
       <c r="X34" s="1">
-        <f>ABS(V34-W34)^1.5</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -3151,7 +3155,7 @@
         <v>-0.17912627790187374</v>
       </c>
       <c r="J35" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,G35:I35)</f>
+        <f t="shared" si="0"/>
         <v>-17.686894168528106</v>
       </c>
       <c r="K35" s="1" cm="1">
@@ -3167,7 +3171,7 @@
         <v>1</v>
       </c>
       <c r="N35" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,K35:M35)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="O35" s="1" cm="1">
@@ -3183,7 +3187,7 @@
         <v>1</v>
       </c>
       <c r="R35" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,O35:Q35)</f>
+        <f t="shared" si="2"/>
         <v>86.08390053389553</v>
       </c>
       <c r="S35" s="1" t="s">
@@ -3203,7 +3207,7 @@
         <v>2</v>
       </c>
       <c r="X35" s="1">
-        <f>ABS(V35-W35)^1.5</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -3239,7 +3243,7 @@
         <v>0.54983805943292885</v>
       </c>
       <c r="J36" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,G36:I36)</f>
+        <f t="shared" si="0"/>
         <v>-18.887908869884448</v>
       </c>
       <c r="K36" s="1" cm="1">
@@ -3255,7 +3259,7 @@
         <v>1</v>
       </c>
       <c r="N36" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,K36:M36)</f>
+        <f t="shared" si="1"/>
         <v>-11.382504941558363</v>
       </c>
       <c r="O36" s="1" cm="1">
@@ -3271,7 +3275,7 @@
         <v>1</v>
       </c>
       <c r="R36" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,O36:Q36)</f>
+        <f t="shared" si="2"/>
         <v>30</v>
       </c>
       <c r="S36" s="1" t="s">
@@ -3291,7 +3295,7 @@
         <v>3</v>
       </c>
       <c r="X36" s="1">
-        <f>ABS(V36-W36)^1.5</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -3327,7 +3331,7 @@
         <v>-0.69289092412419773</v>
       </c>
       <c r="J37" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,G37:I37)</f>
+        <f t="shared" si="0"/>
         <v>-27.264107112719557</v>
       </c>
       <c r="K37" s="1" cm="1">
@@ -3343,7 +3347,7 @@
         <v>0.75574569260534985</v>
       </c>
       <c r="N37" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,K37:M37)</f>
+        <f t="shared" si="1"/>
         <v>-4.7829908056097299</v>
       </c>
       <c r="O37" s="1" cm="1">
@@ -3359,7 +3363,7 @@
         <v>1</v>
       </c>
       <c r="R37" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,O37:Q37)</f>
+        <f t="shared" si="2"/>
         <v>30</v>
       </c>
       <c r="S37" s="1" t="s">
@@ -3381,7 +3385,7 @@
         <v>3</v>
       </c>
       <c r="X37" s="1">
-        <f>ABS(V37-W37)^1.5</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -3417,7 +3421,7 @@
         <v>-1</v>
       </c>
       <c r="J38" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,G38:I38)</f>
+        <f t="shared" si="0"/>
         <v>-27.904149464622073</v>
       </c>
       <c r="K38" s="1" cm="1">
@@ -3433,7 +3437,7 @@
         <v>-0.41622750434489375</v>
       </c>
       <c r="N38" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,K38:M38)</f>
+        <f t="shared" si="1"/>
         <v>-16.31820796907374</v>
       </c>
       <c r="O38" s="1" cm="1">
@@ -3449,7 +3453,7 @@
         <v>1</v>
       </c>
       <c r="R38" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,O38:Q38)</f>
+        <f t="shared" si="2"/>
         <v>83.343544856647043</v>
       </c>
       <c r="S38" s="1" t="s">
@@ -3469,7 +3473,7 @@
         <v>3</v>
       </c>
       <c r="X38" s="1">
-        <f>ABS(V38-W38)^1.5</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -3505,7 +3509,7 @@
         <v>-1</v>
       </c>
       <c r="J39" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,G39:I39)</f>
+        <f t="shared" si="0"/>
         <v>-30</v>
       </c>
       <c r="K39" s="1" cm="1">
@@ -3521,7 +3525,7 @@
         <v>-9.7048070873955727E-2</v>
       </c>
       <c r="N39" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,K39:M39)</f>
+        <f t="shared" si="1"/>
         <v>-16.455721063109337</v>
       </c>
       <c r="O39" s="1" cm="1">
@@ -3537,7 +3541,7 @@
         <v>1</v>
       </c>
       <c r="R39" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,O39:Q39)</f>
+        <f t="shared" si="2"/>
         <v>100</v>
       </c>
       <c r="S39" s="1" t="s">
@@ -3557,7 +3561,7 @@
         <v>3</v>
       </c>
       <c r="X39" s="1">
-        <f>ABS(V39-W39)^1.5</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -3593,7 +3597,7 @@
         <v>-0.31539328776945053</v>
       </c>
       <c r="J40" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,G40:I40)</f>
+        <f t="shared" si="0"/>
         <v>-33.607216811019747</v>
       </c>
       <c r="K40" s="1" cm="1">
@@ -3609,7 +3613,7 @@
         <v>1</v>
       </c>
       <c r="N40" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,K40:M40)</f>
+        <f t="shared" si="1"/>
         <v>-13.123211083078605</v>
       </c>
       <c r="O40" s="1" cm="1">
@@ -3625,7 +3629,7 @@
         <v>1</v>
       </c>
       <c r="R40" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,O40:Q40)</f>
+        <f t="shared" si="2"/>
         <v>30</v>
       </c>
       <c r="S40" s="1" t="s">
@@ -3645,7 +3649,7 @@
         <v>3</v>
       </c>
       <c r="X40" s="1">
-        <f>ABS(V40-W40)^1.5</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -3681,7 +3685,7 @@
         <v>-1</v>
       </c>
       <c r="J41" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,G41:I41)</f>
+        <f t="shared" si="0"/>
         <v>-36.217252978524641</v>
       </c>
       <c r="K41" s="1" cm="1">
@@ -3697,7 +3701,7 @@
         <v>-1</v>
       </c>
       <c r="N41" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,K41:M41)</f>
+        <f t="shared" si="1"/>
         <v>-33.380032912874533</v>
       </c>
       <c r="O41" s="1" cm="1">
@@ -3713,7 +3717,7 @@
         <v>0.36476920729012097</v>
       </c>
       <c r="R41" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,O41:Q41)</f>
+        <f t="shared" si="2"/>
         <v>60.589648032338204</v>
       </c>
       <c r="S41" s="1" t="s">
@@ -3733,7 +3737,7 @@
         <v>3</v>
       </c>
       <c r="X41" s="1">
-        <f>ABS(V41-W41)^1.5</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -3769,7 +3773,7 @@
         <v>-1</v>
       </c>
       <c r="J42" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,G42:I42)</f>
+        <f t="shared" si="0"/>
         <v>-56.754806658911804</v>
       </c>
       <c r="K42" s="1" cm="1">
@@ -3785,7 +3789,7 @@
         <v>-1</v>
       </c>
       <c r="N42" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,K42:M42)</f>
+        <f t="shared" si="1"/>
         <v>-54.670846123589151</v>
       </c>
       <c r="O42" s="1" cm="1">
@@ -3801,7 +3805,7 @@
         <v>-1</v>
       </c>
       <c r="R42" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,O42:Q42)</f>
+        <f t="shared" si="2"/>
         <v>47.368716962397478</v>
       </c>
       <c r="S42" s="1" t="s">
@@ -3821,7 +3825,7 @@
         <v>3</v>
       </c>
       <c r="X42" s="1">
-        <f>ABS(V42-W42)^1.5</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -3857,7 +3861,7 @@
         <v>-0.15242936489198133</v>
       </c>
       <c r="J43" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,G43:I43)</f>
+        <f t="shared" si="0"/>
         <v>-66.914394836901351</v>
       </c>
       <c r="K43" s="1" cm="1">
@@ -3873,7 +3877,7 @@
         <v>1</v>
       </c>
       <c r="N43" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,K43:M43)</f>
+        <f t="shared" si="1"/>
         <v>-48.879019688302748</v>
       </c>
       <c r="O43" s="1" cm="1">
@@ -3889,7 +3893,7 @@
         <v>1</v>
       </c>
       <c r="R43" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,O43:Q43)</f>
+        <f t="shared" si="2"/>
         <v>30</v>
       </c>
       <c r="S43" s="1" t="s">
@@ -3909,7 +3913,7 @@
         <v>3</v>
       </c>
       <c r="X43" s="1">
-        <f>ABS(V43-W43)^1.5</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -3945,7 +3949,7 @@
         <v>0.76362464692458976</v>
       </c>
       <c r="J44" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,G44:I44)</f>
+        <f t="shared" si="0"/>
         <v>-72.189480697075169</v>
       </c>
       <c r="K44" s="1" cm="1">
@@ -3961,7 +3965,7 @@
         <v>1</v>
       </c>
       <c r="N44" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,K44:M44)</f>
+        <f t="shared" si="1"/>
         <v>-67.902477196057987</v>
       </c>
       <c r="O44" s="1" cm="1">
@@ -3977,7 +3981,7 @@
         <v>1</v>
       </c>
       <c r="R44" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,O44:Q44)</f>
+        <f t="shared" si="2"/>
         <v>30</v>
       </c>
       <c r="S44" s="1" t="s">
@@ -3997,7 +4001,7 @@
         <v>3</v>
       </c>
       <c r="X44" s="1">
-        <f>ABS(V44-W44)^1.5</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -4033,7 +4037,7 @@
         <v>-0.48529570746621453</v>
       </c>
       <c r="J45" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,G45:I45)</f>
+        <f t="shared" si="0"/>
         <v>-87.49102805134946</v>
       </c>
       <c r="K45" s="1" cm="1">
@@ -4049,7 +4053,7 @@
         <v>0.96195254991002788</v>
       </c>
       <c r="N45" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,K45:M45)</f>
+        <f t="shared" si="1"/>
         <v>-65.039291728246226</v>
       </c>
       <c r="O45" s="1" cm="1">
@@ -4065,7 +4069,7 @@
         <v>1</v>
       </c>
       <c r="R45" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,O45:Q45)</f>
+        <f t="shared" si="2"/>
         <v>30</v>
       </c>
       <c r="S45" s="1" t="s">
@@ -4085,7 +4089,7 @@
         <v>3</v>
       </c>
       <c r="X45" s="1">
-        <f>ABS(V45-W45)^1.5</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -4121,7 +4125,7 @@
         <v>-1</v>
       </c>
       <c r="J46" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,G46:I46)</f>
+        <f t="shared" si="0"/>
         <v>-89.446626687701269</v>
       </c>
       <c r="K46" s="1" cm="1">
@@ -4137,7 +4141,7 @@
         <v>-1</v>
       </c>
       <c r="N46" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,K46:M46)</f>
+        <f t="shared" si="1"/>
         <v>-88.701132940941235</v>
       </c>
       <c r="O46" s="1" cm="1">
@@ -4153,7 +4157,7 @@
         <v>-1</v>
       </c>
       <c r="R46" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,O46:Q46)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="S46" s="1" t="s">
@@ -4173,7 +4177,7 @@
         <v>3</v>
       </c>
       <c r="X46" s="1">
-        <f>ABS(V46-W46)^1.5</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -4209,7 +4213,7 @@
         <v>-1</v>
       </c>
       <c r="J47" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,G47:I47)</f>
+        <f t="shared" si="0"/>
         <v>-100</v>
       </c>
       <c r="K47" s="1" cm="1">
@@ -4225,7 +4229,7 @@
         <v>-1</v>
       </c>
       <c r="N47" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,K47:M47)</f>
+        <f t="shared" si="1"/>
         <v>-100</v>
       </c>
       <c r="O47" s="1" cm="1">
@@ -4241,7 +4245,7 @@
         <v>0.51459447750570098</v>
       </c>
       <c r="R47" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,O47:Q47)</f>
+        <f t="shared" si="2"/>
         <v>22.718917162585512</v>
       </c>
       <c r="S47" s="1" t="s">
@@ -4261,7 +4265,7 @@
         <v>3</v>
       </c>
       <c r="X47" s="1">
-        <f>ABS(V47-W47)^1.5</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -4297,7 +4301,7 @@
         <v>-1</v>
       </c>
       <c r="J48" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,G48:I48)</f>
+        <f t="shared" si="0"/>
         <v>-100</v>
       </c>
       <c r="K48" s="1" cm="1">
@@ -4313,7 +4317,7 @@
         <v>-1</v>
       </c>
       <c r="N48" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,K48:M48)</f>
+        <f t="shared" si="1"/>
         <v>-100</v>
       </c>
       <c r="O48" s="1" cm="1">
@@ -4329,7 +4333,7 @@
         <v>-1</v>
       </c>
       <c r="R48" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,O48:Q48)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="S48" s="1" t="s">
@@ -4349,7 +4353,7 @@
         <v>3</v>
       </c>
       <c r="X48" s="1">
-        <f>ABS(V48-W48)^1.5</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -4385,7 +4389,7 @@
         <v>-1</v>
       </c>
       <c r="J49" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,G49:I49)</f>
+        <f t="shared" si="0"/>
         <v>-100</v>
       </c>
       <c r="K49" s="1" cm="1">
@@ -4401,7 +4405,7 @@
         <v>-1</v>
       </c>
       <c r="N49" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,K49:M49)</f>
+        <f t="shared" si="1"/>
         <v>-100</v>
       </c>
       <c r="O49" s="1" cm="1">
@@ -4417,7 +4421,7 @@
         <v>-1</v>
       </c>
       <c r="R49" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,O49:Q49)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="S49" s="1" t="s">
@@ -4437,7 +4441,7 @@
         <v>3</v>
       </c>
       <c r="X49" s="1">
-        <f>ABS(V49-W49)^1.5</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -4473,7 +4477,7 @@
         <v>-1</v>
       </c>
       <c r="J50" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,G50:I50)</f>
+        <f t="shared" si="0"/>
         <v>-100</v>
       </c>
       <c r="K50" s="1" cm="1">
@@ -4489,7 +4493,7 @@
         <v>-1</v>
       </c>
       <c r="N50" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,K50:M50)</f>
+        <f t="shared" si="1"/>
         <v>-100</v>
       </c>
       <c r="O50" s="1" cm="1">
@@ -4505,7 +4509,7 @@
         <v>-1</v>
       </c>
       <c r="R50" s="1">
-        <f>SUMPRODUCT($C$10:$E$10,O50:Q50)</f>
+        <f t="shared" si="2"/>
         <v>-100</v>
       </c>
       <c r="S50" s="1" t="s">
@@ -4525,7 +4529,7 @@
         <v>4</v>
       </c>
       <c r="X50" s="1">
-        <f>ABS(V50-W50)^1.5</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -4875,17 +4879,5 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{5513622F-E294-B44C-B206-4A78585D6CC3}">
-          <x14:formula1>
-            <xm:f>#REF!</xm:f>
-          </x14:formula1>
-          <xm:sqref>B6</xm:sqref>
-        </x14:dataValidation>
-      </x14:dataValidations>
-    </ext>
-  </extLst>
 </worksheet>
 </file>
</xml_diff>